<commit_message>
Added few requirements battery management system
</commit_message>
<xml_diff>
--- a/GGVTS/Requirements/exports/srs.xlsx
+++ b/GGVTS/Requirements/exports/srs.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="291">
   <si>
     <t>uid</t>
   </si>
@@ -106,7 +106,7 @@
     <t>1.6</t>
   </si>
   <si>
-    <t>If battery level of GGVTS is less than 5% and host battery level is above hostbatlvltoStartGGVTSchrg GGVTS shall request CM to enable charging for GGVTS battery until GGVTS battery reaches for GGVTSMaxBatteryLvl.</t>
+    <t>If battery level of GGVTS is less than GGVTSbatLvltoStartGGVTS and host battery level is above hostbatlvltoStartGGVTSchrg GGVTS shall request CM to enable charging for GGVTS battery until GGVTS battery reaches for GGVTSMaxBatteryLvl.</t>
   </si>
   <si>
     <t>SRS008</t>
@@ -439,7 +439,7 @@
     <t>5.5</t>
   </si>
   <si>
-    <t>If Condition1 and Condition2 are false, user should be informed as a InformationMessage. Refer SRS128</t>
+    <t>If Condition1 and Condition2 are false, user should be informed as a InformationMessage. Refer Section “Various Message Formats”</t>
   </si>
   <si>
     <t>SRS155</t>
@@ -658,16 +658,367 @@
     <t>Requested functionality "COMMAND"</t>
   </si>
   <si>
+    <t>SRS161</t>
+  </si>
+  <si>
+    <t>VehileBatLow message format</t>
+  </si>
+  <si>
+    <t>SRS162</t>
+  </si>
+  <si>
+    <t>7.6.1</t>
+  </si>
+  <si>
+    <t>Message for VehicleBatLow shall contain following information:</t>
+  </si>
+  <si>
+    <t>SRS163</t>
+  </si>
+  <si>
+    <t>7.6.1.1</t>
+  </si>
+  <si>
+    <t>Text “Vehicle Battery Low Remaining XX%”. Where XX stands for exact percentage of battery level of vehicle.</t>
+  </si>
+  <si>
     <t>SRS158</t>
   </si>
   <si>
+    <t>8</t>
+  </si>
+  <si>
     <t>Waiting for Message</t>
   </si>
   <si>
     <t>SRS160</t>
   </si>
   <si>
+    <t>8.1</t>
+  </si>
+  <si>
     <t>As soon as initialisation finishes, GGVTS shall start waiting for the message.</t>
+  </si>
+  <si>
+    <t>SRS037</t>
+  </si>
+  <si>
+    <t>Battery Management System</t>
+  </si>
+  <si>
+    <t>SRS038</t>
+  </si>
+  <si>
+    <t>Hardware Components</t>
+  </si>
+  <si>
+    <t>SRS039</t>
+  </si>
+  <si>
+    <t>9.1.1</t>
+  </si>
+  <si>
+    <t>Microcontroller PIC16</t>
+  </si>
+  <si>
+    <t>SRS040</t>
+  </si>
+  <si>
+    <t>9.1.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hardware circuitry to provide charge to GGVTS  </t>
+  </si>
+  <si>
+    <t>SRS041</t>
+  </si>
+  <si>
+    <t>Hardware Connections:</t>
+  </si>
+  <si>
+    <t>SRS042</t>
+  </si>
+  <si>
+    <t>BMS shall be connected to GGVTS over SPI.</t>
+  </si>
+  <si>
+    <t>SRS043</t>
+  </si>
+  <si>
+    <t>Inbuilt ADC of BMS shall be connected to vehicle battery.</t>
+  </si>
+  <si>
+    <t>SRS044</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>PIN(TBD)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> shall control relay to start stop charging of GGVTS.</t>
+    </r>
+  </si>
+  <si>
+    <t>SRS046</t>
+  </si>
+  <si>
+    <t>Working of BMS:</t>
+  </si>
+  <si>
+    <t>SRS047</t>
+  </si>
+  <si>
+    <t>Initialisation</t>
+  </si>
+  <si>
+    <t>SRS048</t>
+  </si>
+  <si>
+    <t>Once Power-up, Internal registers related to timers shall get intialized.</t>
+  </si>
+  <si>
+    <t>SRS049</t>
+  </si>
+  <si>
+    <t>Once Power-Up, Internal registers for Interrupts shall e initailized.</t>
+  </si>
+  <si>
+    <t>SRS050</t>
+  </si>
+  <si>
+    <t>Once Power-Up, Internal registers for timer interrupts shall be initialized.</t>
+  </si>
+  <si>
+    <t>SRS051</t>
+  </si>
+  <si>
+    <t>Once Power-Up, Internal registers for SPI shall get initilized.</t>
+  </si>
+  <si>
+    <t>SRS052</t>
+  </si>
+  <si>
+    <t>Once Power-Up, BMS shall act as slave for SPI communication.</t>
+  </si>
+  <si>
+    <t>SRS053</t>
+  </si>
+  <si>
+    <t>Once Power-Up, GGVTS shall act as master for SPI communication.</t>
+  </si>
+  <si>
+    <t>SRS054</t>
+  </si>
+  <si>
+    <t>Once Power-Up, BMS shall perform handshake with GGVTS.</t>
+  </si>
+  <si>
+    <t>SRS055</t>
+  </si>
+  <si>
+    <t>Once Handshake is confirmed and successful, BMS shall go to sleep until and unless its functionality is required by GGVTS.</t>
+  </si>
+  <si>
+    <t>SRS056</t>
+  </si>
+  <si>
+    <t>Sleep State:</t>
+  </si>
+  <si>
+    <t>SRS057</t>
+  </si>
+  <si>
+    <t>Once in sleep, There shall be only two ways to wake BMS up.</t>
+  </si>
+  <si>
+    <t>SRS058</t>
+  </si>
+  <si>
+    <t>1. GGVTS wake BMS up as it needed BMS functionality.</t>
+  </si>
+  <si>
+    <t>SRS059</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">2. If vehicle battery comes equal to or goes down from </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="1"/>
+        <u val="single"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>minBatRequiredtoSelfStart,</t>
+    </r>
+  </si>
+  <si>
+    <t>SRS060</t>
+  </si>
+  <si>
+    <t>Working State:</t>
+  </si>
+  <si>
+    <t>SRS061</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">Software interrupt </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">BatLow </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">shall trigger in GGVTS when battery of GGVTs is lower than </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="1"/>
+        <u val="single"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Ggvtsbatlvltostartggvts.</t>
+    </r>
+  </si>
+  <si>
+    <t>SRS062</t>
+  </si>
+  <si>
+    <t>As soon as BatLow iterrupt occurs. A wake sequence shall be sent to BMS from GGVTS.</t>
+  </si>
+  <si>
+    <t>SRS063</t>
+  </si>
+  <si>
+    <t>When wake up sequence is received by BMS from GGVTS, BMS shall wake up and move to working state.</t>
+  </si>
+  <si>
+    <t>SRS064</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">In working state, BMS shall check for vehicle battery. If vehicle battery is equal or lower than </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="1"/>
+        <u val="single"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>minBatRequiredtoSelfStart,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> GGVTS shall be informed about vehicle battery low event.</t>
+    </r>
+  </si>
+  <si>
+    <t>SRS065</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve">When GGVTs receives vehicle battery low event, A message shall be triggered to user to inform about BatLow event as </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="1"/>
+        <i val="1"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>VehcileBatLow</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t xml:space="preserve"> message and a timer needs to be started for </t>
+    </r>
+    <r>
+      <rPr>
+        <i val="1"/>
+        <u val="single"/>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>timerBatLowwaitforuserresponse</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color indexed="8"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>. Refer section “Various Message Formats”</t>
+    </r>
+  </si>
+  <si>
+    <t>SRS066</t>
+  </si>
+  <si>
+    <t>SRS067</t>
+  </si>
+  <si>
+    <t>SRS068</t>
+  </si>
+  <si>
+    <t>SRS069</t>
   </si>
 </sst>
 </file>
@@ -677,7 +1028,7 @@
   <numFmts count="1">
     <numFmt numFmtId="0" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -695,6 +1046,26 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <u val="single"/>
+      <sz val="11"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
@@ -743,7 +1114,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -761,6 +1132,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" borderId="1" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="left" vertical="bottom"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1842,7 +2222,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:J71"/>
+  <dimension ref="A1:J106"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="9.5" style="1" customWidth="1"/>
@@ -1897,7 +2277,7 @@
       <c r="B2" t="s" s="3">
         <v>11</v>
       </c>
-      <c r="C2" t="s" s="2">
+      <c r="C2" t="s" s="3">
         <v>12</v>
       </c>
       <c r="D2" s="4"/>
@@ -2235,7 +2615,7 @@
       <c r="B15" t="s" s="3">
         <v>51</v>
       </c>
-      <c r="C15" t="s" s="2">
+      <c r="C15" t="s" s="3">
         <v>52</v>
       </c>
       <c r="D15" s="4"/>
@@ -2469,7 +2849,7 @@
       <c r="B24" t="s" s="3">
         <v>78</v>
       </c>
-      <c r="C24" t="s" s="2">
+      <c r="C24" t="s" s="3">
         <v>79</v>
       </c>
       <c r="D24" s="4"/>
@@ -2755,7 +3135,7 @@
       <c r="B35" t="s" s="3">
         <v>111</v>
       </c>
-      <c r="C35" t="s" s="2">
+      <c r="C35" t="s" s="3">
         <v>112</v>
       </c>
       <c r="D35" s="4"/>
@@ -2833,7 +3213,7 @@
       <c r="B38" t="s" s="3">
         <v>120</v>
       </c>
-      <c r="C38" t="s" s="2">
+      <c r="C38" t="s" s="3">
         <v>121</v>
       </c>
       <c r="D38" s="4"/>
@@ -3041,7 +3421,7 @@
       <c r="B46" t="s" s="3">
         <v>144</v>
       </c>
-      <c r="C46" t="s" s="2">
+      <c r="C46" t="s" s="3">
         <v>145</v>
       </c>
       <c r="D46" s="4"/>
@@ -3119,7 +3499,7 @@
       <c r="B49" t="s" s="3">
         <v>153</v>
       </c>
-      <c r="C49" t="s" s="2">
+      <c r="C49" t="s" s="3">
         <v>154</v>
       </c>
       <c r="D49" s="4"/>
@@ -3663,7 +4043,7 @@
         <v>215</v>
       </c>
       <c r="B70" s="5">
-        <v>8</v>
+        <v>7.6</v>
       </c>
       <c r="C70" t="s" s="3">
         <v>216</v>
@@ -3688,11 +4068,11 @@
       <c r="A71" t="s" s="3">
         <v>217</v>
       </c>
-      <c r="B71" s="5">
-        <v>8.1</v>
+      <c r="B71" t="s" s="3">
+        <v>218</v>
       </c>
       <c r="C71" t="s" s="3">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
@@ -3709,6 +4089,788 @@
         <v>1</v>
       </c>
       <c r="J71" s="4"/>
+    </row>
+    <row r="72" ht="26.55" customHeight="1">
+      <c r="A72" t="s" s="3">
+        <v>220</v>
+      </c>
+      <c r="B72" t="s" s="3">
+        <v>221</v>
+      </c>
+      <c r="C72" t="s" s="3">
+        <v>222</v>
+      </c>
+      <c r="D72" s="4"/>
+      <c r="E72" s="4"/>
+      <c r="F72" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G72" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H72" t="s" s="3">
+        <v>220</v>
+      </c>
+      <c r="I72" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J72" s="4"/>
+    </row>
+    <row r="73" ht="13.55" customHeight="1">
+      <c r="A73" t="s" s="3">
+        <v>223</v>
+      </c>
+      <c r="B73" t="s" s="3">
+        <v>224</v>
+      </c>
+      <c r="C73" t="s" s="3">
+        <v>225</v>
+      </c>
+      <c r="D73" s="4"/>
+      <c r="E73" s="4"/>
+      <c r="F73" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G73" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H73" t="s" s="3">
+        <v>225</v>
+      </c>
+      <c r="I73" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J73" s="4"/>
+    </row>
+    <row r="74" ht="13.55" customHeight="1">
+      <c r="A74" t="s" s="3">
+        <v>226</v>
+      </c>
+      <c r="B74" t="s" s="3">
+        <v>227</v>
+      </c>
+      <c r="C74" t="s" s="3">
+        <v>228</v>
+      </c>
+      <c r="D74" s="4"/>
+      <c r="E74" s="4"/>
+      <c r="F74" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G74" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H74" t="s" s="3">
+        <v>226</v>
+      </c>
+      <c r="I74" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J74" s="4"/>
+    </row>
+    <row r="75" ht="13.55" customHeight="1">
+      <c r="A75" t="s" s="3">
+        <v>229</v>
+      </c>
+      <c r="B75" s="5">
+        <v>9</v>
+      </c>
+      <c r="C75" t="s" s="2">
+        <v>230</v>
+      </c>
+      <c r="D75" s="4"/>
+      <c r="E75" s="4"/>
+      <c r="F75" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G75" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H75" t="s" s="3">
+        <v>230</v>
+      </c>
+      <c r="I75" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J75" s="4"/>
+    </row>
+    <row r="76" ht="13.55" customHeight="1">
+      <c r="A76" t="s" s="3">
+        <v>231</v>
+      </c>
+      <c r="B76" s="5">
+        <v>9.1</v>
+      </c>
+      <c r="C76" t="s" s="3">
+        <v>232</v>
+      </c>
+      <c r="D76" s="4"/>
+      <c r="E76" s="4"/>
+      <c r="F76" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G76" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H76" t="s" s="3">
+        <v>231</v>
+      </c>
+      <c r="I76" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J76" s="4"/>
+    </row>
+    <row r="77" ht="13.55" customHeight="1">
+      <c r="A77" t="s" s="3">
+        <v>233</v>
+      </c>
+      <c r="B77" t="s" s="3">
+        <v>234</v>
+      </c>
+      <c r="C77" t="s" s="3">
+        <v>235</v>
+      </c>
+      <c r="D77" s="4"/>
+      <c r="E77" s="4"/>
+      <c r="F77" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G77" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H77" t="s" s="3">
+        <v>233</v>
+      </c>
+      <c r="I77" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J77" s="4"/>
+    </row>
+    <row r="78" ht="13.55" customHeight="1">
+      <c r="A78" t="s" s="3">
+        <v>236</v>
+      </c>
+      <c r="B78" t="s" s="3">
+        <v>237</v>
+      </c>
+      <c r="C78" t="s" s="3">
+        <v>238</v>
+      </c>
+      <c r="D78" s="4"/>
+      <c r="E78" s="4"/>
+      <c r="F78" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G78" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H78" s="4"/>
+      <c r="I78" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J78" s="4"/>
+    </row>
+    <row r="79" ht="13.55" customHeight="1">
+      <c r="A79" t="s" s="3">
+        <v>239</v>
+      </c>
+      <c r="B79" s="4"/>
+      <c r="C79" t="s" s="2">
+        <v>240</v>
+      </c>
+      <c r="D79" s="4"/>
+      <c r="E79" s="4"/>
+      <c r="F79" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G79" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H79" s="4"/>
+      <c r="I79" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J79" s="4"/>
+    </row>
+    <row r="80" ht="13.55" customHeight="1">
+      <c r="A80" t="s" s="3">
+        <v>241</v>
+      </c>
+      <c r="B80" s="4"/>
+      <c r="C80" t="s" s="3">
+        <v>242</v>
+      </c>
+      <c r="D80" s="4"/>
+      <c r="E80" s="4"/>
+      <c r="F80" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G80" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H80" s="4"/>
+      <c r="I80" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J80" s="4"/>
+    </row>
+    <row r="81" ht="13.55" customHeight="1">
+      <c r="A81" t="s" s="3">
+        <v>243</v>
+      </c>
+      <c r="B81" s="4"/>
+      <c r="C81" t="s" s="3">
+        <v>244</v>
+      </c>
+      <c r="D81" s="4"/>
+      <c r="E81" s="4"/>
+      <c r="F81" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G81" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H81" s="4"/>
+      <c r="I81" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J81" s="4"/>
+    </row>
+    <row r="82" ht="13.55" customHeight="1">
+      <c r="A82" t="s" s="3">
+        <v>245</v>
+      </c>
+      <c r="B82" s="4"/>
+      <c r="C82" t="s" s="3">
+        <v>246</v>
+      </c>
+      <c r="D82" s="4"/>
+      <c r="E82" s="4"/>
+      <c r="F82" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G82" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H82" s="4"/>
+      <c r="I82" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J82" s="4"/>
+    </row>
+    <row r="83" ht="13.55" customHeight="1">
+      <c r="A83" t="s" s="3">
+        <v>247</v>
+      </c>
+      <c r="B83" s="6"/>
+      <c r="C83" t="s" s="7">
+        <v>248</v>
+      </c>
+      <c r="D83" s="6"/>
+      <c r="E83" s="6"/>
+      <c r="F83" t="b" s="8">
+        <v>1</v>
+      </c>
+      <c r="G83" t="b" s="8">
+        <v>0</v>
+      </c>
+      <c r="H83" s="6"/>
+      <c r="I83" t="b" s="8">
+        <v>1</v>
+      </c>
+      <c r="J83" s="6"/>
+    </row>
+    <row r="84" ht="13.55" customHeight="1">
+      <c r="A84" t="s" s="3">
+        <v>249</v>
+      </c>
+      <c r="B84" s="4"/>
+      <c r="C84" t="s" s="2">
+        <v>250</v>
+      </c>
+      <c r="D84" s="4"/>
+      <c r="E84" s="4"/>
+      <c r="F84" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G84" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H84" s="4"/>
+      <c r="I84" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J84" s="4"/>
+    </row>
+    <row r="85" ht="13.55" customHeight="1">
+      <c r="A85" t="s" s="3">
+        <v>251</v>
+      </c>
+      <c r="B85" s="4"/>
+      <c r="C85" t="s" s="3">
+        <v>252</v>
+      </c>
+      <c r="D85" s="4"/>
+      <c r="E85" s="4"/>
+      <c r="F85" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G85" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H85" s="4"/>
+      <c r="I85" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J85" s="4"/>
+    </row>
+    <row r="86" ht="13.55" customHeight="1">
+      <c r="A86" t="s" s="3">
+        <v>253</v>
+      </c>
+      <c r="B86" s="4"/>
+      <c r="C86" t="s" s="3">
+        <v>254</v>
+      </c>
+      <c r="D86" s="4"/>
+      <c r="E86" s="4"/>
+      <c r="F86" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G86" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H86" s="4"/>
+      <c r="I86" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J86" s="4"/>
+    </row>
+    <row r="87" ht="13.55" customHeight="1">
+      <c r="A87" t="s" s="3">
+        <v>255</v>
+      </c>
+      <c r="B87" s="4"/>
+      <c r="C87" t="s" s="3">
+        <v>256</v>
+      </c>
+      <c r="D87" s="4"/>
+      <c r="E87" s="4"/>
+      <c r="F87" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G87" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H87" s="4"/>
+      <c r="I87" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J87" s="4"/>
+    </row>
+    <row r="88" ht="13.55" customHeight="1">
+      <c r="A88" t="s" s="3">
+        <v>257</v>
+      </c>
+      <c r="B88" s="4"/>
+      <c r="C88" t="s" s="3">
+        <v>258</v>
+      </c>
+      <c r="D88" s="4"/>
+      <c r="E88" s="4"/>
+      <c r="F88" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G88" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H88" s="4"/>
+      <c r="I88" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J88" s="4"/>
+    </row>
+    <row r="89" ht="13.55" customHeight="1">
+      <c r="A89" t="s" s="3">
+        <v>259</v>
+      </c>
+      <c r="B89" s="4"/>
+      <c r="C89" t="s" s="3">
+        <v>260</v>
+      </c>
+      <c r="D89" s="4"/>
+      <c r="E89" s="4"/>
+      <c r="F89" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G89" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H89" s="4"/>
+      <c r="I89" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J89" s="4"/>
+    </row>
+    <row r="90" ht="13.55" customHeight="1">
+      <c r="A90" t="s" s="3">
+        <v>261</v>
+      </c>
+      <c r="B90" s="4"/>
+      <c r="C90" t="s" s="3">
+        <v>262</v>
+      </c>
+      <c r="D90" s="4"/>
+      <c r="E90" s="4"/>
+      <c r="F90" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G90" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H90" s="4"/>
+      <c r="I90" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J90" s="4"/>
+    </row>
+    <row r="91" ht="13.55" customHeight="1">
+      <c r="A91" t="s" s="3">
+        <v>263</v>
+      </c>
+      <c r="B91" s="4"/>
+      <c r="C91" t="s" s="3">
+        <v>264</v>
+      </c>
+      <c r="D91" s="4"/>
+      <c r="E91" s="4"/>
+      <c r="F91" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G91" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H91" s="4"/>
+      <c r="I91" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J91" s="4"/>
+    </row>
+    <row r="92" ht="26.55" customHeight="1">
+      <c r="A92" t="s" s="3">
+        <v>265</v>
+      </c>
+      <c r="B92" s="4"/>
+      <c r="C92" t="s" s="3">
+        <v>266</v>
+      </c>
+      <c r="D92" s="4"/>
+      <c r="E92" s="4"/>
+      <c r="F92" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G92" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H92" s="4"/>
+      <c r="I92" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J92" s="4"/>
+    </row>
+    <row r="93" ht="13.55" customHeight="1">
+      <c r="A93" t="s" s="3">
+        <v>267</v>
+      </c>
+      <c r="B93" s="4"/>
+      <c r="C93" t="s" s="2">
+        <v>268</v>
+      </c>
+      <c r="D93" s="4"/>
+      <c r="E93" s="4"/>
+      <c r="F93" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G93" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H93" s="4"/>
+      <c r="I93" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J93" s="4"/>
+    </row>
+    <row r="94" ht="13.55" customHeight="1">
+      <c r="A94" t="s" s="3">
+        <v>269</v>
+      </c>
+      <c r="B94" s="4"/>
+      <c r="C94" t="s" s="3">
+        <v>270</v>
+      </c>
+      <c r="D94" s="4"/>
+      <c r="E94" s="4"/>
+      <c r="F94" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G94" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H94" s="4"/>
+      <c r="I94" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J94" s="4"/>
+    </row>
+    <row r="95" ht="13.55" customHeight="1">
+      <c r="A95" t="s" s="3">
+        <v>271</v>
+      </c>
+      <c r="B95" s="4"/>
+      <c r="C95" t="s" s="3">
+        <v>272</v>
+      </c>
+      <c r="D95" s="4"/>
+      <c r="E95" s="4"/>
+      <c r="F95" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G95" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H95" s="4"/>
+      <c r="I95" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J95" s="4"/>
+    </row>
+    <row r="96" ht="13.55" customHeight="1">
+      <c r="A96" t="s" s="3">
+        <v>273</v>
+      </c>
+      <c r="B96" s="4"/>
+      <c r="C96" t="s" s="3">
+        <v>274</v>
+      </c>
+      <c r="D96" s="4"/>
+      <c r="E96" s="4"/>
+      <c r="F96" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G96" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H96" s="4"/>
+      <c r="I96" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J96" s="4"/>
+    </row>
+    <row r="97" ht="13.55" customHeight="1">
+      <c r="A97" t="s" s="3">
+        <v>275</v>
+      </c>
+      <c r="B97" s="4"/>
+      <c r="C97" t="s" s="2">
+        <v>276</v>
+      </c>
+      <c r="D97" s="4"/>
+      <c r="E97" s="4"/>
+      <c r="F97" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G97" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H97" s="4"/>
+      <c r="I97" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J97" s="4"/>
+    </row>
+    <row r="98" ht="26.55" customHeight="1">
+      <c r="A98" t="s" s="3">
+        <v>277</v>
+      </c>
+      <c r="B98" s="4"/>
+      <c r="C98" t="s" s="3">
+        <v>278</v>
+      </c>
+      <c r="D98" s="4"/>
+      <c r="E98" s="4"/>
+      <c r="F98" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G98" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H98" s="4"/>
+      <c r="I98" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J98" s="4"/>
+    </row>
+    <row r="99" ht="26.55" customHeight="1">
+      <c r="A99" t="s" s="3">
+        <v>279</v>
+      </c>
+      <c r="B99" s="4"/>
+      <c r="C99" t="s" s="3">
+        <v>280</v>
+      </c>
+      <c r="D99" s="4"/>
+      <c r="E99" s="4"/>
+      <c r="F99" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G99" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H99" s="4"/>
+      <c r="I99" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J99" s="4"/>
+    </row>
+    <row r="100" ht="26.55" customHeight="1">
+      <c r="A100" t="s" s="3">
+        <v>281</v>
+      </c>
+      <c r="B100" s="4"/>
+      <c r="C100" t="s" s="3">
+        <v>282</v>
+      </c>
+      <c r="D100" s="4"/>
+      <c r="E100" s="4"/>
+      <c r="F100" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G100" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H100" s="4"/>
+      <c r="I100" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J100" s="4"/>
+    </row>
+    <row r="101" ht="39.55" customHeight="1">
+      <c r="A101" t="s" s="3">
+        <v>283</v>
+      </c>
+      <c r="B101" s="4"/>
+      <c r="C101" t="s" s="3">
+        <v>284</v>
+      </c>
+      <c r="D101" s="4"/>
+      <c r="E101" s="4"/>
+      <c r="F101" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G101" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H101" s="4"/>
+      <c r="I101" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J101" s="4"/>
+    </row>
+    <row r="102" ht="52.55" customHeight="1">
+      <c r="A102" t="s" s="3">
+        <v>285</v>
+      </c>
+      <c r="B102" s="4"/>
+      <c r="C102" t="s" s="3">
+        <v>286</v>
+      </c>
+      <c r="D102" s="4"/>
+      <c r="E102" s="4"/>
+      <c r="F102" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G102" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H102" s="4"/>
+      <c r="I102" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J102" s="4"/>
+    </row>
+    <row r="103" ht="13.55" customHeight="1">
+      <c r="A103" t="s" s="3">
+        <v>287</v>
+      </c>
+      <c r="B103" s="4"/>
+      <c r="C103" s="4"/>
+      <c r="D103" s="4"/>
+      <c r="E103" s="4"/>
+      <c r="F103" s="4"/>
+      <c r="G103" s="4"/>
+      <c r="H103" s="4"/>
+      <c r="I103" s="4"/>
+      <c r="J103" s="4"/>
+    </row>
+    <row r="104" ht="13.55" customHeight="1">
+      <c r="A104" t="s" s="3">
+        <v>288</v>
+      </c>
+      <c r="B104" s="4"/>
+      <c r="C104" s="4"/>
+      <c r="D104" s="4"/>
+      <c r="E104" s="4"/>
+      <c r="F104" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G104" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H104" s="4"/>
+      <c r="I104" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J104" s="4"/>
+    </row>
+    <row r="105" ht="13.55" customHeight="1">
+      <c r="A105" t="s" s="3">
+        <v>289</v>
+      </c>
+      <c r="B105" s="4"/>
+      <c r="C105" s="4"/>
+      <c r="D105" s="4"/>
+      <c r="E105" s="4"/>
+      <c r="F105" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G105" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H105" s="4"/>
+      <c r="I105" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J105" s="4"/>
+    </row>
+    <row r="106" ht="13.55" customHeight="1">
+      <c r="A106" t="s" s="3">
+        <v>290</v>
+      </c>
+      <c r="B106" s="4"/>
+      <c r="C106" s="4"/>
+      <c r="D106" s="4"/>
+      <c r="E106" s="4"/>
+      <c r="F106" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="G106" t="b" s="5">
+        <v>0</v>
+      </c>
+      <c r="H106" s="4"/>
+      <c r="I106" t="b" s="5">
+        <v>1</v>
+      </c>
+      <c r="J106" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>